<commit_message>
osbservation_utility excel files, naming update (no underscores)
</commit_message>
<xml_diff>
--- a/ai4sh/import_data/utility/observation/excel/analysis_method.xlsx
+++ b/ai4sh/import_data/utility/observation/excel/analysis_method.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="204">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -73,7 +73,7 @@
     <t xml:space="preserve">Optical emission spectroscopy</t>
   </si>
   <si>
-    <t xml:space="preserve">usda_caco3</t>
+    <t xml:space="preserve">usda caco3</t>
   </si>
   <si>
     <t xml:space="preserve">CaCO&lt;sub&gt;3&lt;/sub&gt; (USDA)</t>
@@ -103,6 +103,9 @@
     <t xml:space="preserve">volumetric method, calcimeter back titration with HCl, sample sieved&lt;2mm base </t>
   </si>
   <si>
+    <t xml:space="preserve">usda a273</t>
+  </si>
+  <si>
     <t xml:space="preserve">usda_a273</t>
   </si>
   <si>
@@ -118,7 +121,10 @@
     <t xml:space="preserve">11260:1994</t>
   </si>
   <si>
-    <t xml:space="preserve">usda_cf</t>
+    <t xml:space="preserve">usda cf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USDA coarse fraction</t>
   </si>
   <si>
     <t xml:space="preserve">c236</t>
@@ -133,7 +139,10 @@
     <t xml:space="preserve">11464:2006</t>
   </si>
   <si>
-    <t xml:space="preserve">usda_clay</t>
+    <t xml:space="preserve">usda clay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USDA clay</t>
   </si>
   <si>
     <t xml:space="preserve">a334</t>
@@ -151,7 +160,10 @@
     <t xml:space="preserve">Laser diffraction, sample sieved&lt;2 mm base</t>
   </si>
   <si>
-    <t xml:space="preserve">usda_ec</t>
+    <t xml:space="preserve">usda ec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USDA electrical conductivity</t>
   </si>
   <si>
     <t xml:space="preserve">a364</t>
@@ -169,7 +181,10 @@
     <t xml:space="preserve">Extraction with a barium chloride solution buffered at pH 8.2 and ICP-OES (Inductively Coupled Plasma Optical Emission Spectrometry)</t>
   </si>
   <si>
-    <t xml:space="preserve">usda_k-ext</t>
+    <t xml:space="preserve">usda k-ext</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USDA extractable Potassium</t>
   </si>
   <si>
     <t xml:space="preserve">a725</t>
@@ -196,7 +211,7 @@
     <t xml:space="preserve">11885:2007</t>
   </si>
   <si>
-    <t xml:space="preserve">usda_n-tot</t>
+    <t xml:space="preserve">usda n-tot</t>
   </si>
   <si>
     <t xml:space="preserve">a263</t>
@@ -259,7 +274,10 @@
     <t xml:space="preserve">11260:2021</t>
   </si>
   <si>
-    <t xml:space="preserve">usda_soc</t>
+    <t xml:space="preserve">usda soc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USDA Soil Organic Carbon (SOC)</t>
   </si>
   <si>
     <t xml:space="preserve">c729</t>
@@ -277,7 +295,10 @@
     <t xml:space="preserve">0.5 M bicarbonate extraction and spectroscopy (Olsen method)</t>
   </si>
   <si>
-    <t xml:space="preserve">usda_p-ext</t>
+    <t xml:space="preserve">usda p-ext</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USDA extractable Phosphorus</t>
   </si>
   <si>
     <t xml:space="preserve">a274</t>
@@ -295,7 +316,10 @@
     <t xml:space="preserve">0.01 M CaCl2 at a 1:2 soil:solution ratio</t>
   </si>
   <si>
-    <t xml:space="preserve">usda_ph-cacl2</t>
+    <t xml:space="preserve">usda ph-cacl2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USDA pH(CaCl&lt;sub&gt;2&lt;/sub&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">a481</t>
@@ -391,6 +415,45 @@
     <t xml:space="preserve">Undisturbed soil sample taken in a cylinder of known volume dried at 105 C, bulk density is the net weight of the dried soil divided by the cylinder volume.</t>
   </si>
   <si>
+    <t xml:space="preserve">ai4sh prokaryotes metabarcoding bioinfo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI4SH prokaryotes metabarcoding bioinfo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://ai4sh.github.io/in-situ_data_docs/docs/in-situ_methods/edna/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extraction (ZymoBIOMICS DNA Miniprep Kit), forward amplification (515f Modified GTGYCAGCMGCCGCGGTAA), reverse amplification (806r Modified GGACTACNVGGGTWTCTAAT), purification (magnetic bead), sequencing (platform: Illumina; strategy: 2x250; data requirement: 30K tags), reference library (Silva), bioinformatics(Qiime2-DADA2, FLASH, vsearch package)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai4sh fungi metabarcoding bioinfo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI4SH fungi metabarcoding bioinfo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extraction (ymoBIOMICS DNA Miniprep Kit), forward amplification (515f Modified GTGYCAGCMGCCGCGGTAA), reverse amplification (806r Modified GGACTACNVGGGTWTCTAAT), purification (magnetic bead), sequencing (platform: Illumina; strategy: 2x250; data requirement: 30K tags), reference library (Silva), bioinformatics(Qiime2-DADA2, FLASH, vsearch package), functional prediction (Faprotax), nucleotide sequence library (Sequence Read Archive)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai4sh prokaryotes metabarcoding function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI4SH prokaryotes metabarcoding function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extraction (ymoBIOMICS DNA Miniprep Kit), forward amplification (gITS7 GTGARTCATCGARTCTTTG), reverse amplification (ITS4 TCCTCCGCTTATTGATATGC), purification (magnetic bead), sequencing (platform: Illumina; strategy: 2x250; data requirement: 30K tags), reference library (Unite), bioinformatics(Qiime2-DADA2, FLASH, vsearch package)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai4sh fungi metabarcoding function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI4SH fungi metabarcoding function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extraction (ymoBIOMICS DNA Miniprep Kit), forward amplification (gITS7 GTGARTCATCGARTCTTTG), reverse amplification (ITS4 TCCTCCGCTTATTGATATGC), purification (magnetic bead), sequencing (platform: Illumina; strategy: 2x250; data requirement: 30K tags), reference library (Unite), bioinformatics(Qiime2-DADA2, FLASH, vsearch package), functional prediction (Fungild), nucleotide sequence library (Sequence Read Archive)</t>
+  </si>
+  <si>
     <t xml:space="preserve">beerkan estimation of soil transfer parameters</t>
   </si>
   <si>
@@ -547,13 +610,19 @@
     <t xml:space="preserve">Exchangable cations ammonium acetate</t>
   </si>
   <si>
+    <t xml:space="preserve">derived</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Derived</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Derived nominative classification from one or more numerical values</t>
+  </si>
+  <si>
     <t xml:space="preserve">ai4sh 16s metabarcoding</t>
   </si>
   <si>
     <t xml:space="preserve">AI4SH 16s metabarcoding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extraction (ZymoBIOMICS DNA Miniprep Kit), forward amplification (515f Modified GTGYCAGCMGCCGCGGTAA), reverse amplification (806r Modified GGACTACNVGGGTWTCTAAT), purification (magnetic bead), sequencing (platform: Illumina; strategy: 2x250; data requirement: 30K tags), reference library (Silva), bioinformatics(Qiime2-DADA2, FLASH, vsearch package)</t>
   </si>
   <si>
     <t xml:space="preserve">ai4sh its metabarcoding</t>
@@ -573,7 +642,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="[hh]:mm:ss"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -618,7 +687,19 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -666,7 +747,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -675,7 +756,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -696,6 +777,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -886,7 +975,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.44"/>
@@ -895,10 +984,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.72"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="8" style="2" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="8" style="1" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -917,8 +1006,9 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -934,8 +1024,10 @@
       <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -951,8 +1043,10 @@
       <c r="E3" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -968,8 +1062,10 @@
       <c r="E4" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -985,8 +1081,10 @@
       <c r="E5" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1002,8 +1100,10 @@
       <c r="E6" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -1022,8 +1122,9 @@
       <c r="F7" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>22</v>
       </c>
@@ -1042,630 +1143,663 @@
       <c r="F8" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>30</v>
+      </c>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>30</v>
+      </c>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>42</v>
+      </c>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>45</v>
+      </c>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>49</v>
+      </c>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>52</v>
+      </c>
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>56</v>
+      </c>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>59</v>
+      </c>
+      <c r="G18" s="1"/>
+    </row>
+    <row r="19" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+    </row>
+    <row r="20" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>65</v>
+      </c>
+      <c r="G20" s="1"/>
+    </row>
+    <row r="21" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>68</v>
+      </c>
+      <c r="G21" s="1"/>
+    </row>
+    <row r="22" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>71</v>
+      </c>
+      <c r="G22" s="1"/>
+    </row>
+    <row r="23" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>74</v>
+      </c>
+      <c r="G23" s="1"/>
+    </row>
+    <row r="24" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+      <c r="G24" s="1"/>
+    </row>
+    <row r="25" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+      <c r="G25" s="1"/>
+    </row>
+    <row r="26" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+      <c r="G26" s="1"/>
+    </row>
+    <row r="27" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+      <c r="G27" s="1"/>
+    </row>
+    <row r="28" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>87</v>
+      </c>
+      <c r="G28" s="1"/>
+    </row>
+    <row r="29" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F29" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F29" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="G29" s="1"/>
+    </row>
+    <row r="30" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>94</v>
+      </c>
+      <c r="G30" s="1"/>
+    </row>
+    <row r="31" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>97</v>
+      </c>
+      <c r="G31" s="1"/>
+    </row>
+    <row r="32" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>97</v>
+      </c>
+      <c r="G32" s="1"/>
+    </row>
+    <row r="33" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>45</v>
+      </c>
+      <c r="G33" s="1"/>
+    </row>
+    <row r="34" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>45</v>
+      </c>
+      <c r="G34" s="1"/>
+    </row>
+    <row r="35" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>45</v>
+      </c>
+      <c r="G35" s="1"/>
+    </row>
+    <row r="36" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>45</v>
+      </c>
+      <c r="G36" s="1"/>
+    </row>
+    <row r="37" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>107</v>
+      </c>
+      <c r="G37" s="1"/>
+    </row>
+    <row r="38" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>107</v>
+      </c>
+      <c r="G38" s="1"/>
+    </row>
+    <row r="39" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>107</v>
+      </c>
+      <c r="G39" s="1"/>
+    </row>
+    <row r="40" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>8</v>
@@ -1677,15 +1811,16 @@
         <v>8</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>111</v>
+      </c>
+      <c r="G40" s="1"/>
+    </row>
+    <row r="41" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>8</v>
@@ -1697,15 +1832,16 @@
         <v>8</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>114</v>
+      </c>
+      <c r="G41" s="1"/>
+    </row>
+    <row r="42" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>8</v>
@@ -1717,15 +1853,16 @@
         <v>8</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>114</v>
+      </c>
+      <c r="G42" s="1"/>
+    </row>
+    <row r="43" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>8</v>
@@ -1737,15 +1874,16 @@
         <v>8</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>119</v>
+      </c>
+      <c r="G43" s="1"/>
+    </row>
+    <row r="44" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>8</v>
@@ -1757,15 +1895,16 @@
         <v>8</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>119</v>
+      </c>
+      <c r="G44" s="1"/>
+    </row>
+    <row r="45" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>8</v>
@@ -1777,15 +1916,16 @@
         <v>8</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>124</v>
+      </c>
+      <c r="G45" s="1"/>
+    </row>
+    <row r="46" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>8</v>
@@ -1797,15 +1937,16 @@
         <v>8</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>127</v>
+      </c>
+      <c r="G46" s="1"/>
+    </row>
+    <row r="47" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>8</v>
@@ -1817,15 +1958,16 @@
         <v>8</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>130</v>
+      </c>
+      <c r="G47" s="1"/>
+    </row>
+    <row r="48" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>8</v>
@@ -1834,18 +1976,19 @@
         <v>8</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>134</v>
+      </c>
+      <c r="G48" s="1"/>
+    </row>
+    <row r="49" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>8</v>
@@ -1854,18 +1997,19 @@
         <v>8</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>8</v>
+        <v>133</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>137</v>
+      </c>
+      <c r="G49" s="1"/>
+    </row>
+    <row r="50" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>8</v>
@@ -1874,367 +2018,490 @@
         <v>8</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>8</v>
+        <v>133</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="G50" s="1"/>
+    </row>
+    <row r="51" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E51" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B51" s="7" t="s">
+      <c r="F51" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="G51" s="1"/>
+    </row>
+    <row r="52" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="G52" s="1"/>
+    </row>
+    <row r="53" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="G53" s="1"/>
+    </row>
+    <row r="54" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="G54" s="1"/>
+    </row>
+    <row r="55" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F55" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="G55" s="1"/>
+    </row>
+    <row r="56" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+    </row>
+    <row r="57" s="2" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="G57" s="1"/>
+    </row>
+    <row r="58" s="2" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="G58" s="1"/>
+    </row>
+    <row r="59" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G59" s="1"/>
+    </row>
+    <row r="60" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G60" s="1"/>
+    </row>
+    <row r="61" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="G61" s="1"/>
+    </row>
+    <row r="62" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F62" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="G62" s="1"/>
+    </row>
+    <row r="63" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="G63" s="1"/>
+    </row>
+    <row r="64" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="G64" s="1"/>
+    </row>
+    <row r="65" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="G65" s="1"/>
+    </row>
+    <row r="66" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="G66" s="1"/>
+    </row>
+    <row r="67" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="G67" s="1"/>
+    </row>
+    <row r="68" s="2" customFormat="true" ht="14.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B68" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D68" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="G68" s="1"/>
+    </row>
+    <row r="69" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="G69" s="1"/>
+    </row>
+    <row r="70" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="G70" s="1"/>
+    </row>
+    <row r="71" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="G71" s="1"/>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F72" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C51" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F51" s="7" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="B58" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F58" s="7" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F61" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="14.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="B64" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D64" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E67" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F67" s="1" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D68" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E68" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F68" s="1" t="s">
-        <v>180</v>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>